<commit_message>
Increased Wait Timeout for Start Planning CTA
</commit_message>
<xml_diff>
--- a/Data/Failed.xlsx
+++ b/Data/Failed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>*** Test Cases ***</t>
   </si>
@@ -43,41 +43,17 @@
     <t>${expectedCremationNoFacilities}</t>
   </si>
   <si>
-    <t>https://staging.altogetherfuneral.com/funeral-cremation/california/placerville/el-dorado-funeral-cremation-services-placerville/caaed.html?_vis_preview_data=eyJhIjoiYTE1MTUyYWNhY2I2MTU2ZDJlZWQxNzRlZmFkYjhmMWMiLCJlIjp7IjEzOCI6eyJ2IjoiMSIsImQiOjAsInMiOjAsInRnIjowLCJ0IjowLCJ0ZCI6MCwibCI6MCwiYWxoIjowLCJpcGxlIjowLCJpaG8iOjAsInBhaGkiOm51bGwsInNhYmVyIjpudWxsLCJuZXdRdWVyeUJveCI6bnVsbCwiZGF0YVJlZ2lvbiI6bnVsbCwibWF0Y2hUeXBlIjpudWxsLCJjbiI6InVuZGVmaW5lZCIsInVybCI6Imh0dHBzJTI1M0ElMjUyRiUyNTJGc3RhZ2luZy5hbHRvZ2V0aGVyZnVuZXJhbC5jb20lMjUyRmZ1bmVyYWwtY3JlbWF0aW9uJTI1MkZhcml6b25hJTI1MkZtb2hhdmUtdmFsbGV5JTI1MkZkZXNlcnQtbGF3bi1mdW5lcmFsLWhvbWUtbW9oYXZlJTI1MkZhenNkbS5odG1sIiwiYXBwIjoiYXBwIiwidHMiOjE3NjEwNTQwMzMwNDJ9fX0=</t>
-  </si>
-  <si>
-    <t>caaed</t>
-  </si>
-  <si>
-    <t>https://staging.altogetherfuneral.com/funeral-cremation/california/pine-grove/amador-hills-cremation-funeral-service/cadll.html?_vis_preview_data=eyJhIjoiYTE1MTUyYWNhY2I2MTU2ZDJlZWQxNzRlZmFkYjhmMWMiLCJlIjp7IjEyNiI6eyJ2IjoiMSIsImQiOjAsInMiOjAsInRnIjowLCJ0IjowLCJ0ZCI6MCwibCI6MCwiYWxoIjowLCJpcGxlIjowLCJpaG8iOjAsInBhaGkiOm51bGwsInNhYmVyIjpudWxsLCJuZXdRdWVyeUJveCI6bnVsbCwiZGF0YVJlZ2lvbiI6bnVsbCwibWF0Y2hUeXBlIjpudWxsLCJjbiI6InVuZGVmaW5lZCIsInVybCI6Imh0dHBzJTI1M0ElMjUyRiUyNTJGZGV2ZWxvcG1lbnQuYWx0b2dldGhlcmZ1bmVyYWwuY29tJTI1MkZmdW5lcmFsLWNyZW1hdGlvbiUyNTJGbmV3LXlvcmslMjUyRmFtc3RlcmRhbSUyNTJGYmV0ei1yb3NzaS1iZWxsaW5nZXItc3Rld2FydC1hbXN0ZXJkYW0lMjUyRm55YW1zLmh0bWwiLCJhcHAiOiJhcHAiLCJ0cyI6MTc1NzQwNzIzNzk2MH19fQ==</t>
-  </si>
-  <si>
-    <t>cadll</t>
-  </si>
-  <si>
-    <t>https://staging.altogetherfuneral.com/funeral-cremation/oregon/molalla/molalla-funeral-chapel/orcmf.html</t>
-  </si>
-  <si>
-    <t>orcmf</t>
-  </si>
-  <si>
-    <t>https://staging.altogetherfuneral.com/funeral-cremation/oregon/salem/crown-cremation-services-salem/orcms.html?_vis_preview_data=eyJhIjoiYTE1MTUyYWNhY2I2MTU2ZDJlZWQxNzRlZmFkYjhmMWMiLCJlIjp7IjEyNiI6eyJ2IjoiMSIsImQiOjAsInMiOjAsInRnIjowLCJ0IjowLCJ0ZCI6MCwibCI6MCwiYWxoIjowLCJpcGxlIjowLCJpaG8iOjAsInBhaGkiOm51bGwsInNhYmVyIjpudWxsLCJuZXdRdWVyeUJveCI6bnVsbCwiZGF0YVJlZ2lvbiI6bnVsbCwibWF0Y2hUeXBlIjpudWxsLCJjbiI6InVuZGVmaW5lZCIsInVybCI6Imh0dHBzJTI1M0ElMjUyRiUyNTJGZGV2ZWxvcG1lbnQuYWx0b2dldGhlcmZ1bmVyYWwuY29tJTI1MkZmdW5lcmFsLWNyZW1hdGlvbiUyNTJGbmV3LXlvcmslMjUyRmFtc3RlcmRhbSUyNTJGYmV0ei1yb3NzaS1iZWxsaW5nZXItc3Rld2FydC1hbXN0ZXJkYW0lMjUyRm55YW1zLmh0bWwiLCJhcHAiOiJhcHAiLCJ0cyI6MTc1NzQwNzIzNzk2MH19fQ==</t>
-  </si>
-  <si>
-    <t>orcms</t>
-  </si>
-  <si>
-    <t>https://staging.altogetherfuneral.com/funeral-cremation/oregon/tualatin/crown-cremation-services-tualatin/orcmt.html?_vis_preview_data=eyJhIjoiYTE1MTUyYWNhY2I2MTU2ZDJlZWQxNzRlZmFkYjhmMWMiLCJlIjp7IjEyNiI6eyJ2IjoiMSIsImQiOjAsInMiOjAsInRnIjowLCJ0IjowLCJ0ZCI6MCwibCI6MCwiYWxoIjowLCJpcGxlIjowLCJpaG8iOjAsInBhaGkiOm51bGwsInNhYmVyIjpudWxsLCJuZXdRdWVyeUJveCI6bnVsbCwiZGF0YVJlZ2lvbiI6bnVsbCwibWF0Y2hUeXBlIjpudWxsLCJjbiI6InVuZGVmaW5lZCIsInVybCI6Imh0dHBzJTI1M0ElMjUyRiUyNTJGZGV2ZWxvcG1lbnQuYWx0b2dldGhlcmZ1bmVyYWwuY29tJTI1MkZmdW5lcmFsLWNyZW1hdGlvbiUyNTJGbmV3LXlvcmslMjUyRmFtc3RlcmRhbSUyNTJGYmV0ei1yb3NzaS1iZWxsaW5nZXItc3Rld2FydC1hbXN0ZXJkYW0lMjUyRm55YW1zLmh0bWwiLCJhcHAiOiJhcHAiLCJ0cyI6MTc1NzQwNzIzNzk2MH19fQ==</t>
-  </si>
-  <si>
-    <t>orcmt</t>
+    <t>https://staging.altogetherfuneral.com/funeral-cremation/arizona/phoenix/samaritan-funeral-cremation-services/azsfp.html</t>
+  </si>
+  <si>
+    <t>azsfp</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -92,24 +68,13 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFD966"/>
-        <bgColor rgb="FFFFD966"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -118,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -131,16 +96,13 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -394,8 +356,8 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="str">
-        <f t="shared" ref="A2:A6" si="1">"Run GS for "&amp;C2</f>
-        <v>Run GS for caaed</v>
+        <f>"Run GS for "&amp;C2</f>
+        <v>Run GS for azsfp</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>10</v>
@@ -426,141 +388,54 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Run GS for cadll</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E3" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="F3" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="G3" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="H3" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="I3" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="J3" s="5">
-        <v>3.0</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Run GS for orcmf</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="F4" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="G4" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="H4" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="I4" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="J4" s="5">
-        <v>3.0</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Run GS for orcms</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E5" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="G5" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="H5" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="I5" s="5">
-        <v>4.0</v>
-      </c>
-      <c r="J5" s="5">
-        <v>3.0</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>Run GS for orcmt</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E6" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="F6" s="5">
-        <v>0.0</v>
-      </c>
-      <c r="G6" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="H6" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="I6" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="J6" s="5">
-        <v>3.0</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="B2"/>
-  </hyperlinks>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>